<commit_message>
[FIX] Generate reports & Month Selector
</commit_message>
<xml_diff>
--- a/public/plantilla_materia_prima.xlsx
+++ b/public/plantilla_materia_prima.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luisi\OneDrive\Escritorio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2457F335-F201-4636-98AA-B2C5CE8A0D61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CF906EA-3125-45AC-87FE-E1CAC052CA3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
-  <si>
-    <t>Fecha ingreso</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
   <si>
     <t>Descripción</t>
   </si>
@@ -43,13 +40,10 @@
     <t>Observaciones</t>
   </si>
   <si>
-    <t>m</t>
+    <t>mm</t>
   </si>
   <si>
     <t>Ejemplo</t>
-  </si>
-  <si>
-    <t>00/00/2025</t>
   </si>
 </sst>
 </file>
@@ -108,12 +102,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -421,14 +412,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -446,34 +437,37 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2">
+      <c r="E2">
         <v>0</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>7</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1:D1048576" xr:uid="{D41DB9A0-9546-4744-AC81-20B3C89887D3}">
+      <formula1>"mm, cm, m, mg, g, kg, ml, L, Pieza, Caja, Rollo, Paquete, Bolsa, Docena, Unidad, Par, Set"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C1048576" xr:uid="{7B3EF160-C37B-4D54-8AB6-0C2B1B5F32AA}">
+      <formula1>0</formula1>
+      <formula2>5000</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>